<commit_message>
release latest solvency workflow and Step7 updates
</commit_message>
<xml_diff>
--- a/config/solvency_company_urls.xlsx
+++ b/config/solvency_company_urls.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\KPMG\Solvency_Report_System\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3D54BBC-72F8-4F35-9683-5B4778A9D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03399DC-F121-4552-B504-3E9A92958A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="公司网址" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterate="1" calcOnSave="0" concurrentManualCount="32"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -578,10 +578,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>https://www.picc.com.cn/xwzx/gkxx/zxxx/jtcfnl/</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>https://www.abchinalife.com/xxpl/zxxx/cfnljdpl/index.shtml</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
@@ -603,6 +599,10 @@
   </si>
   <si>
     <t>https://www.tianan-life.com/toGongKaiXinXiPiLu.html</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.picc-pension.com.cn/html/category/2304/20030-1.htm</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -774,11 +774,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -801,13 +801,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="SolvencyCompanyUrls" displayName="SolvencyCompanyUrls" ref="A3:C95" totalsRowShown="0">
-  <autoFilter ref="A3:C95" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="珠江人寿"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A3:C95" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="公司"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="公司类别"/>
@@ -1021,11 +1015,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
@@ -1038,7 +1032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1">
+    <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -1049,7 +1043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1">
+    <row r="5" spans="1:3">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
@@ -1060,7 +1054,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1">
+    <row r="6" spans="1:3">
       <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
@@ -1071,7 +1065,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1">
+    <row r="7" spans="1:3">
       <c r="A7" s="5" t="s">
         <v>11</v>
       </c>
@@ -1082,7 +1076,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1">
+    <row r="8" spans="1:3">
       <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
@@ -1093,7 +1087,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1">
+    <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
         <v>15</v>
       </c>
@@ -1104,7 +1098,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1">
+    <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
         <v>17</v>
       </c>
@@ -1115,7 +1109,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1">
+    <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
         <v>19</v>
       </c>
@@ -1126,7 +1120,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1">
+    <row r="12" spans="1:3">
       <c r="A12" s="5" t="s">
         <v>21</v>
       </c>
@@ -1137,7 +1131,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1">
+    <row r="13" spans="1:3">
       <c r="A13" s="5" t="s">
         <v>23</v>
       </c>
@@ -1148,7 +1142,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1">
+    <row r="14" spans="1:3">
       <c r="A14" s="5" t="s">
         <v>25</v>
       </c>
@@ -1159,7 +1153,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1">
+    <row r="15" spans="1:3">
       <c r="A15" s="5" t="s">
         <v>27</v>
       </c>
@@ -1170,7 +1164,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1">
+    <row r="16" spans="1:3">
       <c r="A16" s="5" t="s">
         <v>29</v>
       </c>
@@ -1181,7 +1175,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1">
+    <row r="17" spans="1:3">
       <c r="A17" s="5" t="s">
         <v>31</v>
       </c>
@@ -1192,7 +1186,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1">
+    <row r="18" spans="1:3">
       <c r="A18" s="5" t="s">
         <v>33</v>
       </c>
@@ -1203,7 +1197,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="28" hidden="1">
+    <row r="19" spans="1:3" ht="28">
       <c r="A19" s="5" t="s">
         <v>35</v>
       </c>
@@ -1214,7 +1208,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1">
+    <row r="20" spans="1:3">
       <c r="A20" s="5" t="s">
         <v>37</v>
       </c>
@@ -1225,7 +1219,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1">
+    <row r="21" spans="1:3">
       <c r="A21" s="5" t="s">
         <v>39</v>
       </c>
@@ -1236,7 +1230,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1">
+    <row r="22" spans="1:3">
       <c r="A22" s="5" t="s">
         <v>41</v>
       </c>
@@ -1247,7 +1241,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1">
+    <row r="23" spans="1:3">
       <c r="A23" s="5" t="s">
         <v>43</v>
       </c>
@@ -1258,18 +1252,18 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1">
+    <row r="24" spans="1:3">
       <c r="A24" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="11" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1">
+    <row r="25" spans="1:3">
       <c r="A25" s="5" t="s">
         <v>46</v>
       </c>
@@ -1280,7 +1274,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1">
+    <row r="26" spans="1:3">
       <c r="A26" s="5" t="s">
         <v>48</v>
       </c>
@@ -1291,7 +1285,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1">
+    <row r="27" spans="1:3">
       <c r="A27" s="5" t="s">
         <v>50</v>
       </c>
@@ -1302,7 +1296,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1">
+    <row r="28" spans="1:3">
       <c r="A28" s="5" t="s">
         <v>52</v>
       </c>
@@ -1313,7 +1307,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1">
+    <row r="29" spans="1:3">
       <c r="A29" s="5" t="s">
         <v>54</v>
       </c>
@@ -1324,7 +1318,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1">
+    <row r="30" spans="1:3">
       <c r="A30" s="5" t="s">
         <v>56</v>
       </c>
@@ -1335,7 +1329,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1">
+    <row r="31" spans="1:3">
       <c r="A31" s="5" t="s">
         <v>58</v>
       </c>
@@ -1346,18 +1340,18 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="28" hidden="1">
+    <row r="32" spans="1:3" ht="28">
       <c r="A32" s="5" t="s">
         <v>60</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="11" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1">
+    <row r="33" spans="1:3">
       <c r="A33" s="5" t="s">
         <v>61</v>
       </c>
@@ -1368,7 +1362,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1">
+    <row r="34" spans="1:3">
       <c r="A34" s="5" t="s">
         <v>63</v>
       </c>
@@ -1379,7 +1373,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="28" hidden="1">
+    <row r="35" spans="1:3" ht="28">
       <c r="A35" s="5" t="s">
         <v>65</v>
       </c>
@@ -1390,7 +1384,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="28" hidden="1">
+    <row r="36" spans="1:3" ht="28">
       <c r="A36" s="5" t="s">
         <v>67</v>
       </c>
@@ -1401,18 +1395,18 @@
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1">
+    <row r="37" spans="1:3">
       <c r="A37" s="5" t="s">
         <v>69</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="11" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1">
+    <row r="38" spans="1:3">
       <c r="A38" s="5" t="s">
         <v>70</v>
       </c>
@@ -1423,7 +1417,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="42" hidden="1">
+    <row r="39" spans="1:3" ht="42">
       <c r="A39" s="5" t="s">
         <v>72</v>
       </c>
@@ -1434,7 +1428,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1">
+    <row r="40" spans="1:3">
       <c r="A40" s="5" t="s">
         <v>74</v>
       </c>
@@ -1445,7 +1439,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:3" hidden="1">
+    <row r="41" spans="1:3">
       <c r="A41" s="5" t="s">
         <v>76</v>
       </c>
@@ -1456,7 +1450,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1">
+    <row r="42" spans="1:3">
       <c r="A42" s="5" t="s">
         <v>78</v>
       </c>
@@ -1467,7 +1461,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1">
+    <row r="43" spans="1:3">
       <c r="A43" s="5" t="s">
         <v>80</v>
       </c>
@@ -1478,7 +1472,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="28" hidden="1">
+    <row r="44" spans="1:3" ht="28">
       <c r="A44" s="5" t="s">
         <v>82</v>
       </c>
@@ -1489,7 +1483,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1">
+    <row r="45" spans="1:3">
       <c r="A45" s="5" t="s">
         <v>84</v>
       </c>
@@ -1500,7 +1494,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" spans="1:3" hidden="1">
+    <row r="46" spans="1:3">
       <c r="A46" s="5" t="s">
         <v>86</v>
       </c>
@@ -1511,7 +1505,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="47" spans="1:3" hidden="1">
+    <row r="47" spans="1:3">
       <c r="A47" s="5" t="s">
         <v>88</v>
       </c>
@@ -1522,7 +1516,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:3" hidden="1">
+    <row r="48" spans="1:3">
       <c r="A48" s="5" t="s">
         <v>91</v>
       </c>
@@ -1533,7 +1527,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="49" spans="1:3" hidden="1">
+    <row r="49" spans="1:3">
       <c r="A49" s="5" t="s">
         <v>94</v>
       </c>
@@ -1544,7 +1538,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1">
+    <row r="50" spans="1:3">
       <c r="A50" s="5" t="s">
         <v>96</v>
       </c>
@@ -1555,7 +1549,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="51" spans="1:3" hidden="1">
+    <row r="51" spans="1:3">
       <c r="A51" s="5" t="s">
         <v>98</v>
       </c>
@@ -1566,29 +1560,29 @@
         <v>99</v>
       </c>
     </row>
-    <row r="52" spans="1:3" hidden="1">
+    <row r="52" spans="1:3">
       <c r="A52" s="5" t="s">
         <v>100</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="C52" s="11" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="53" spans="1:3" hidden="1">
+    <row r="53" spans="1:3">
       <c r="A53" s="5" t="s">
         <v>101</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C53" s="12" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" hidden="1">
+      <c r="C53" s="11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
       <c r="A54" s="5" t="s">
         <v>102</v>
       </c>
@@ -1599,7 +1593,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="55" spans="1:3" hidden="1">
+    <row r="55" spans="1:3">
       <c r="A55" s="5" t="s">
         <v>104</v>
       </c>
@@ -1610,7 +1604,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="56" spans="1:3" hidden="1">
+    <row r="56" spans="1:3">
       <c r="A56" s="5" t="s">
         <v>106</v>
       </c>
@@ -1621,7 +1615,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="57" spans="1:3" hidden="1">
+    <row r="57" spans="1:3">
       <c r="A57" s="5" t="s">
         <v>108</v>
       </c>
@@ -1632,7 +1626,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="58" spans="1:3" hidden="1">
+    <row r="58" spans="1:3">
       <c r="A58" s="5" t="s">
         <v>110</v>
       </c>
@@ -1643,7 +1637,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="59" spans="1:3" hidden="1">
+    <row r="59" spans="1:3">
       <c r="A59" s="5" t="s">
         <v>112</v>
       </c>
@@ -1654,7 +1648,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="60" spans="1:3" hidden="1">
+    <row r="60" spans="1:3">
       <c r="A60" s="5" t="s">
         <v>114</v>
       </c>
@@ -1665,7 +1659,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="61" spans="1:3" hidden="1">
+    <row r="61" spans="1:3">
       <c r="A61" s="5" t="s">
         <v>116</v>
       </c>
@@ -1676,7 +1670,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="42" hidden="1">
+    <row r="62" spans="1:3" ht="42">
       <c r="A62" s="5" t="s">
         <v>118</v>
       </c>
@@ -1687,7 +1681,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="63" spans="1:3" hidden="1">
+    <row r="63" spans="1:3">
       <c r="A63" s="5" t="s">
         <v>120</v>
       </c>
@@ -1698,7 +1692,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="64" spans="1:3" hidden="1">
+    <row r="64" spans="1:3">
       <c r="A64" s="5" t="s">
         <v>122</v>
       </c>
@@ -1709,7 +1703,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="65" spans="1:3" hidden="1">
+    <row r="65" spans="1:3">
       <c r="A65" s="5" t="s">
         <v>124</v>
       </c>
@@ -1720,18 +1714,18 @@
         <v>125</v>
       </c>
     </row>
-    <row r="66" spans="1:3" hidden="1">
+    <row r="66" spans="1:3">
       <c r="A66" s="5" t="s">
         <v>126</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C66" s="12" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" ht="28" hidden="1">
+      <c r="C66" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="28">
       <c r="A67" s="5" t="s">
         <v>127</v>
       </c>
@@ -1742,7 +1736,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="68" spans="1:3" hidden="1">
+    <row r="68" spans="1:3">
       <c r="A68" s="5" t="s">
         <v>129</v>
       </c>
@@ -1753,18 +1747,18 @@
         <v>130</v>
       </c>
     </row>
-    <row r="69" spans="1:3" hidden="1">
+    <row r="69" spans="1:3">
       <c r="A69" s="5" t="s">
         <v>131</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C69" s="12" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" hidden="1">
+      <c r="C69" s="11" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
       <c r="A70" s="5" t="s">
         <v>132</v>
       </c>
@@ -1775,18 +1769,18 @@
         <v>133</v>
       </c>
     </row>
-    <row r="71" spans="1:3" hidden="1">
+    <row r="71" spans="1:3">
       <c r="A71" s="5" t="s">
         <v>134</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C71" s="12" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" hidden="1">
+      <c r="C71" s="11" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
       <c r="A72" s="5" t="s">
         <v>135</v>
       </c>
@@ -1797,7 +1791,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="73" spans="1:3" hidden="1">
+    <row r="73" spans="1:3">
       <c r="A73" s="5" t="s">
         <v>137</v>
       </c>
@@ -1808,7 +1802,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="74" spans="1:3" hidden="1">
+    <row r="74" spans="1:3">
       <c r="A74" s="5" t="s">
         <v>139</v>
       </c>
@@ -1819,7 +1813,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="75" spans="1:3" hidden="1">
+    <row r="75" spans="1:3">
       <c r="A75" s="5" t="s">
         <v>141</v>
       </c>
@@ -1830,7 +1824,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="76" spans="1:3" hidden="1">
+    <row r="76" spans="1:3">
       <c r="A76" s="5" t="s">
         <v>143</v>
       </c>
@@ -1841,7 +1835,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="77" spans="1:3" hidden="1">
+    <row r="77" spans="1:3">
       <c r="A77" s="5" t="s">
         <v>145</v>
       </c>
@@ -1852,29 +1846,29 @@
         <v>146</v>
       </c>
     </row>
-    <row r="78" spans="1:3" hidden="1">
+    <row r="78" spans="1:3">
       <c r="A78" s="5" t="s">
         <v>147</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C78" s="12" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" hidden="1">
+      <c r="C78" s="11" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
       <c r="A79" s="5" t="s">
         <v>148</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C79" s="12" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" hidden="1">
+      <c r="C79" s="11" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
       <c r="A80" s="5" t="s">
         <v>149</v>
       </c>
@@ -1885,7 +1879,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="81" spans="1:3" hidden="1">
+    <row r="81" spans="1:3">
       <c r="A81" s="5" t="s">
         <v>151</v>
       </c>
@@ -1896,7 +1890,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="82" spans="1:3" hidden="1">
+    <row r="82" spans="1:3">
       <c r="A82" s="5" t="s">
         <v>153</v>
       </c>
@@ -1907,7 +1901,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="83" spans="1:3" hidden="1">
+    <row r="83" spans="1:3">
       <c r="A83" s="5" t="s">
         <v>155</v>
       </c>
@@ -1918,7 +1912,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="84" spans="1:3" hidden="1">
+    <row r="84" spans="1:3">
       <c r="A84" s="5" t="s">
         <v>157</v>
       </c>
@@ -1929,7 +1923,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="28" hidden="1">
+    <row r="85" spans="1:3" ht="28">
       <c r="A85" s="5" t="s">
         <v>159</v>
       </c>
@@ -1940,7 +1934,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="86" spans="1:3" hidden="1">
+    <row r="86" spans="1:3">
       <c r="A86" s="5" t="s">
         <v>161</v>
       </c>
@@ -1951,7 +1945,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="87" spans="1:3" hidden="1">
+    <row r="87" spans="1:3">
       <c r="A87" s="5" t="s">
         <v>163</v>
       </c>
@@ -1962,7 +1956,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="88" spans="1:3" hidden="1">
+    <row r="88" spans="1:3">
       <c r="A88" s="5" t="s">
         <v>165</v>
       </c>
@@ -1973,7 +1967,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="89" spans="1:3" hidden="1">
+    <row r="89" spans="1:3">
       <c r="A89" s="5" t="s">
         <v>167</v>
       </c>
@@ -1984,18 +1978,18 @@
         <v>168</v>
       </c>
     </row>
-    <row r="90" spans="1:3" hidden="1">
+    <row r="90" spans="1:3">
       <c r="A90" s="5" t="s">
         <v>169</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C90" s="12" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" hidden="1">
+      <c r="C90" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3">
       <c r="A91" s="5" t="s">
         <v>170</v>
       </c>
@@ -2013,11 +2007,11 @@
       <c r="B92" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C92" s="12" t="s">
+      <c r="C92" s="11" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="93" spans="1:3" hidden="1">
+    <row r="93" spans="1:3">
       <c r="A93" s="5" t="s">
         <v>174</v>
       </c>
@@ -2028,7 +2022,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="94" spans="1:3" hidden="1">
+    <row r="94" spans="1:3">
       <c r="A94" s="5" t="s">
         <v>176</v>
       </c>
@@ -2039,7 +2033,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="28" hidden="1">
+    <row r="95" spans="1:3" ht="28">
       <c r="A95" s="6" t="s">
         <v>178</v>
       </c>

</xml_diff>